<commit_message>
HWZ Unterlagen for 2026
</commit_message>
<xml_diff>
--- a/Mathe_Uebungen/Bremskurve.xlsx
+++ b/Mathe_Uebungen/Bremskurve.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Landwirtschaft\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Landwirtschaft\Documents\SoruceCode\Mathe_Uebungen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EDF4CED-DB6D-4FE0-A745-475445B8D221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8181352F-FB7E-4E4C-A465-01CCC4614F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BB21B76C-7116-46E2-A7EB-6C8E623491A5}"/>
   </bookViews>
@@ -350,7 +350,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -470,7 +470,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>30</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>10</c:v>
@@ -689,13 +689,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>-50</c:v>
+                  <c:v>-25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>100</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>250</c:v>
+                  <c:v>125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -852,6 +852,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -859,7 +860,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1492,9 +1492,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1532,7 +1532,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1638,7 +1638,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1780,7 +1780,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1812,7 +1812,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="20">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D5" s="21">
         <v>10</v>
@@ -1889,15 +1889,15 @@
       </c>
       <c r="C16" s="18">
         <f>$C$27*C14+$C$28</f>
-        <v>-50</v>
+        <v>-25</v>
       </c>
       <c r="D16" s="18">
         <f t="shared" ref="D16:E16" si="1">$C$27*D14+$C$28</f>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E16" s="19">
         <f t="shared" si="1"/>
-        <v>250</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="21" x14ac:dyDescent="0.5">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="C27" s="15">
         <f>($C$6-$D$6)/($C$5-$D$5)</f>
-        <v>5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="C28" s="24">
         <f>C6-C27*C5</f>
-        <v>-50</v>
+        <v>-25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>